<commit_message>
Add provider-neutral password field to tracker
</commit_message>
<xml_diff>
--- a/docs/open-brain-credential-tracker.xlsx
+++ b/docs/open-brain-credential-tracker.xlsx
@@ -740,7 +740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.5" customWidth="1" style="33" min="1" max="1"/>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D24" s="46" t="inlineStr">
         <is>
-          <t>AI Provider Account Email / Login</t>
+          <t>AI Provider Account Email</t>
         </is>
       </c>
       <c r="E24" s="47" t="n"/>
@@ -1057,135 +1057,132 @@
       </c>
       <c r="D25" s="46" t="inlineStr">
         <is>
+          <t>AI Provider Account Password / Login Method</t>
+        </is>
+      </c>
+      <c r="E25" s="47" t="n"/>
+    </row>
+    <row r="26" ht="30" customHeight="1" s="34">
+      <c r="B26" s="44" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C26" s="45" t="inlineStr">
+        <is>
+          <t>ENTER</t>
+        </is>
+      </c>
+      <c r="D26" s="46" t="inlineStr">
+        <is>
           <t>AI API Key</t>
         </is>
       </c>
-      <c r="E25" s="47" t="n"/>
-    </row>
-    <row r="26" ht="7.5" customHeight="1" s="34"/>
-    <row r="27" ht="31.5" customHeight="1" s="34">
-      <c r="A27" s="57" t="n"/>
-      <c r="B27" s="58" t="inlineStr">
+      <c r="E26" s="47" t="n"/>
+    </row>
+    <row r="27" ht="31.5" customHeight="1" s="34"/>
+    <row r="28" ht="21.75" customHeight="1" s="34">
+      <c r="A28" s="57" t="n"/>
+      <c r="B28" s="58" t="inlineStr">
         <is>
           <t>STEP 5 — CREATE AN ACCESS KEY</t>
         </is>
       </c>
-      <c r="F27" s="57" t="n"/>
-    </row>
-    <row r="28" ht="21.75" customHeight="1" s="34">
-      <c r="B28" s="42" t="inlineStr">
+      <c r="F28" s="57" t="n"/>
+    </row>
+    <row r="29" ht="30" customHeight="1" s="34">
+      <c r="B29" s="42" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C28" s="42" t="inlineStr">
+      <c r="C29" s="42" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D28" s="43" t="inlineStr">
+      <c r="D29" s="43" t="inlineStr">
         <is>
           <t>What</t>
         </is>
       </c>
-      <c r="E28" s="43" t="inlineStr">
+      <c r="E29" s="43" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="30" customHeight="1" s="34">
-      <c r="B29" s="44" t="inlineStr">
+    <row r="30" ht="7.5" customHeight="1" s="34">
+      <c r="B30" s="44" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C29" s="45" t="inlineStr">
+      <c r="C30" s="45" t="inlineStr">
         <is>
           <t>ENTER</t>
         </is>
       </c>
-      <c r="D29" s="46" t="inlineStr">
+      <c r="D30" s="46" t="inlineStr">
         <is>
           <t>MCP Access Key (output of openssl rand -hex 32)</t>
         </is>
       </c>
-      <c r="E29" s="47" t="n"/>
-    </row>
-    <row r="30" ht="7.5" customHeight="1" s="34"/>
-    <row r="31" ht="31.5" customHeight="1" s="34">
-      <c r="A31" s="59" t="n"/>
-      <c r="B31" s="60" t="inlineStr">
+      <c r="E30" s="47" t="n"/>
+    </row>
+    <row r="31" ht="31.5" customHeight="1" s="34"/>
+    <row r="32" ht="21.75" customHeight="1" s="34">
+      <c r="A32" s="59" t="n"/>
+      <c r="B32" s="60" t="inlineStr">
         <is>
           <t>STEP 6 — DEPLOY THE MCP SERVER</t>
         </is>
       </c>
-      <c r="F31" s="59" t="n"/>
-    </row>
-    <row r="32" ht="21.75" customHeight="1" s="34">
-      <c r="B32" s="42" t="inlineStr">
+      <c r="F32" s="59" t="n"/>
+    </row>
+    <row r="33" ht="30" customHeight="1" s="34">
+      <c r="B33" s="42" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C32" s="42" t="inlineStr">
+      <c r="C33" s="42" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D32" s="43" t="inlineStr">
+      <c r="D33" s="43" t="inlineStr">
         <is>
           <t>What</t>
         </is>
       </c>
-      <c r="E32" s="43" t="inlineStr">
+      <c r="E33" s="43" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="30" customHeight="1" s="34">
-      <c r="B33" s="44" t="inlineStr">
+    <row r="34" ht="30" customHeight="1" s="34">
+      <c r="B34" s="44" t="inlineStr">
         <is>
           <t>6.4</t>
         </is>
       </c>
-      <c r="C33" s="61" t="inlineStr">
+      <c r="C34" s="61" t="inlineStr">
         <is>
           <t>COPY</t>
         </is>
       </c>
-      <c r="D33" s="46" t="inlineStr">
+      <c r="D34" s="46" t="inlineStr">
         <is>
           <t>Terminal: supabase link command</t>
         </is>
       </c>
-      <c r="E33" s="62">
+      <c r="E34" s="62">
         <f>IF(E11="","← enter Project Ref in Step 1","supabase link --project-ref "&amp;E11)</f>
         <v/>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1" s="34">
-      <c r="B34" s="44" t="inlineStr">
-        <is>
-          <t>6.5</t>
-        </is>
-      </c>
-      <c r="C34" s="61" t="inlineStr">
-        <is>
-          <t>COPY</t>
-        </is>
-      </c>
-      <c r="D34" s="46" t="inlineStr">
-        <is>
-          <t>Terminal: set MCP Access Key secret</t>
-        </is>
-      </c>
-      <c r="E34" s="62">
-        <f>IF(E29="","← enter Access Key in Step 5","supabase secrets set MCP_ACCESS_KEY="&amp;E29)</f>
-        <v/>
-      </c>
-    </row>
     <row r="35" ht="30" customHeight="1" s="34">
       <c r="B35" s="44" t="inlineStr">
         <is>
@@ -1199,113 +1196,113 @@
       </c>
       <c r="D35" s="46" t="inlineStr">
         <is>
-          <t>Terminal: set AI API Key secret</t>
+          <t>Terminal: set MCP Access Key secret</t>
         </is>
       </c>
       <c r="E35" s="62">
-        <f>IF(E25="","← enter AI API Key in Step 4",IF(E23="","← enter Provider in Step 4",IF(ISNUMBER(SEARCH("openai",LOWER(E23))),"supabase secrets set OPENAI_API_KEY="&amp;E25,"supabase secrets set OPENROUTER_API_KEY="&amp;E25)))</f>
+        <f>IF(E30="","← enter Access Key in Step 5","supabase secrets set MCP_ACCESS_KEY="&amp;E30)</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1" s="34">
       <c r="B36" s="44" t="inlineStr">
         <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="C36" s="61" t="inlineStr">
+        <is>
+          <t>COPY</t>
+        </is>
+      </c>
+      <c r="D36" s="46" t="inlineStr">
+        <is>
+          <t>Terminal: set AI API Key secret</t>
+        </is>
+      </c>
+      <c r="E36" s="62">
+        <f>IF(E26="","← enter AI API Key in Step 4",IF(E23="","← enter Provider in Step 4",IF(ISNUMBER(SEARCH("openai",LOWER(E23))),"supabase secrets set OPENAI_API_KEY="&amp;E26,"supabase secrets set OPENROUTER_API_KEY="&amp;E26)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1" s="34">
+      <c r="B37" s="44" t="inlineStr">
+        <is>
           <t>6.7</t>
         </is>
       </c>
-      <c r="C36" s="53" t="inlineStr">
+      <c r="C37" s="53" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="D36" s="46" t="inlineStr">
+      <c r="D37" s="46" t="inlineStr">
         <is>
           <t>MCP Server URL</t>
         </is>
       </c>
-      <c r="E36" s="54">
+      <c r="E37" s="54">
         <f>IF(E11="","← enter Project Ref in Step 1","https://"&amp;E11&amp;".supabase.co/functions/v1/open-brain-mcp")</f>
         <v/>
       </c>
     </row>
-    <row r="37" ht="30" customHeight="1" s="34">
-      <c r="B37" s="44" t="inlineStr">
+    <row r="38" ht="7.5" customHeight="1" s="34">
+      <c r="B38" s="44" t="inlineStr">
         <is>
           <t>6.7</t>
         </is>
       </c>
-      <c r="C37" s="53" t="inlineStr">
+      <c r="C38" s="53" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="D37" s="46" t="inlineStr">
+      <c r="D38" s="46" t="inlineStr">
         <is>
           <t>MCP Connection URL</t>
         </is>
       </c>
-      <c r="E37" s="54">
-        <f>IF(OR(E11="",E29=""),"← enter Project Ref + Access Key","https://"&amp;E11&amp;".supabase.co/functions/v1/open-brain-mcp?key="&amp;E29)</f>
+      <c r="E38" s="54">
+        <f>IF(OR(E11="",E30=""),"← enter Project Ref + Access Key","https://"&amp;E11&amp;".supabase.co/functions/v1/open-brain-mcp?key="&amp;E30)</f>
         <v/>
       </c>
     </row>
-    <row r="38" ht="7.5" customHeight="1" s="34"/>
-    <row r="39" ht="31.5" customHeight="1" s="34">
-      <c r="A39" s="63" t="n"/>
-      <c r="B39" s="64" t="inlineStr">
+    <row r="39" ht="31.5" customHeight="1" s="34"/>
+    <row r="40" ht="21.75" customHeight="1" s="34">
+      <c r="A40" s="63" t="n"/>
+      <c r="B40" s="64" t="inlineStr">
         <is>
           <t>STEP 7 — CONNECT TO YOUR AI</t>
         </is>
       </c>
-      <c r="F39" s="63" t="n"/>
-    </row>
-    <row r="40" ht="21.75" customHeight="1" s="34">
-      <c r="B40" s="42" t="inlineStr">
+      <c r="F40" s="63" t="n"/>
+    </row>
+    <row r="41" ht="30" customHeight="1" s="34">
+      <c r="B41" s="42" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C40" s="42" t="inlineStr">
+      <c r="C41" s="42" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D40" s="43" t="inlineStr">
+      <c r="D41" s="43" t="inlineStr">
         <is>
           <t>What</t>
         </is>
       </c>
-      <c r="E40" s="43" t="inlineStr">
+      <c r="E41" s="43" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
-      </c>
-    </row>
-    <row r="41" ht="30" customHeight="1" s="34">
-      <c r="B41" s="44" t="inlineStr">
-        <is>
-          <t>7.1</t>
-        </is>
-      </c>
-      <c r="C41" s="61" t="inlineStr">
-        <is>
-          <t>COPY</t>
-        </is>
-      </c>
-      <c r="D41" s="46" t="inlineStr">
-        <is>
-          <t>Claude Desktop → Connectors → Remote MCP server URL</t>
-        </is>
-      </c>
-      <c r="E41" s="62">
-        <f>E37</f>
-        <v/>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1" s="34">
       <c r="B42" s="44" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C42" s="61" t="inlineStr">
@@ -1315,18 +1312,18 @@
       </c>
       <c r="D42" s="46" t="inlineStr">
         <is>
-          <t>ChatGPT → Apps &amp; Connectors → MCP endpoint URL</t>
+          <t>Claude Desktop → Connectors → Remote MCP server URL</t>
         </is>
       </c>
       <c r="E42" s="62">
-        <f>E37</f>
+        <f>E38</f>
         <v/>
       </c>
     </row>
     <row r="43" ht="36" customHeight="1" s="34">
       <c r="B43" s="44" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="C43" s="61" t="inlineStr">
@@ -1336,45 +1333,66 @@
       </c>
       <c r="D43" s="46" t="inlineStr">
         <is>
-          <t>Terminal: Claude Code CLI command</t>
+          <t>ChatGPT → Apps &amp; Connectors → MCP endpoint URL</t>
         </is>
       </c>
       <c r="E43" s="62">
-        <f>IF(OR(E11="",E29=""),"← enter Project Ref + Access Key","claude mcp add --transport http open-brain https://"&amp;E11&amp;".supabase.co/functions/v1/open-brain-mcp --header "&amp;CHAR(34)&amp;"x-brain-key: "&amp;E29&amp;CHAR(34))</f>
+        <f>E38</f>
         <v/>
       </c>
     </row>
     <row r="44" ht="219.75" customHeight="1" s="34">
       <c r="B44" s="44" t="inlineStr">
         <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="C44" s="61" t="inlineStr">
+        <is>
+          <t>COPY</t>
+        </is>
+      </c>
+      <c r="D44" s="46" t="inlineStr">
+        <is>
+          <t>Terminal: Claude Code CLI command</t>
+        </is>
+      </c>
+      <c r="E44" s="62">
+        <f>IF(OR(E11="",E30=""),"← enter Project Ref + Access Key","claude mcp add --transport http open-brain https://"&amp;E11&amp;".supabase.co/functions/v1/open-brain-mcp --header "&amp;CHAR(34)&amp;"x-brain-key: "&amp;E30&amp;CHAR(34))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="7.5" customHeight="1" s="34">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
           <t>7.4</t>
         </is>
       </c>
-      <c r="C44" s="61" t="inlineStr">
+      <c r="C45" s="61" t="inlineStr">
         <is>
           <t>COPY</t>
         </is>
       </c>
-      <c r="D44" s="46" t="inlineStr">
+      <c r="D45" s="46" t="inlineStr">
         <is>
           <t>JSON config for mcp-remote clients
 (Cursor, VS Code, Windsurf)</t>
         </is>
       </c>
-      <c r="E44" s="62">
-        <f>IF(OR(E11="",E29=""),"← enter Project Ref + Access Key","{" &amp; CHAR(10)&amp; "  " &amp; CHAR(34) &amp; "mcpServers" &amp; CHAR(34) &amp; ": {" &amp; CHAR(10)&amp; "    " &amp; CHAR(34) &amp; "open-brain" &amp; CHAR(34) &amp; ": {" &amp; CHAR(10)&amp; "      " &amp; CHAR(34) &amp; "command" &amp; CHAR(34) &amp; ": " &amp; CHAR(34) &amp; "npx" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "      " &amp; CHAR(34) &amp; "args" &amp; CHAR(34) &amp; ": [" &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "mcp-remote" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "https://" &amp; E11 &amp; ".supabase.co/functions/v1/open-brain-mcp" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "--header" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "x-brain-key:${BRAIN_KEY}" &amp; CHAR(34) &amp; CHAR(10)&amp; "      ]," &amp; CHAR(10)&amp; "      " &amp; CHAR(34) &amp; "env" &amp; CHAR(34) &amp; ": {" &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "BRAIN_KEY" &amp; CHAR(34) &amp; ": " &amp; CHAR(34) &amp; E29 &amp; CHAR(34) &amp; CHAR(10)&amp; "      }" &amp; CHAR(10)&amp; "    }" &amp; CHAR(10)&amp; "  }" &amp; CHAR(10)&amp; "}")</f>
+      <c r="E45" s="62">
+        <f>IF(OR(E11="",E30=""),"← enter Project Ref + Access Key","{" &amp; CHAR(10)&amp; "  " &amp; CHAR(34) &amp; "mcpServers" &amp; CHAR(34) &amp; ": {" &amp; CHAR(10)&amp; "    " &amp; CHAR(34) &amp; "open-brain" &amp; CHAR(34) &amp; ": {" &amp; CHAR(10)&amp; "      " &amp; CHAR(34) &amp; "command" &amp; CHAR(34) &amp; ": " &amp; CHAR(34) &amp; "npx" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "      " &amp; CHAR(34) &amp; "args" &amp; CHAR(34) &amp; ": [" &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "mcp-remote" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "https://" &amp; E11 &amp; ".supabase.co/functions/v1/open-brain-mcp" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "--header" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "x-brain-key:${BRAIN_KEY}" &amp; CHAR(34) &amp; CHAR(10)&amp; "      ]," &amp; CHAR(10)&amp; "      " &amp; CHAR(34) &amp; "env" &amp; CHAR(34) &amp; ": {" &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "BRAIN_KEY" &amp; CHAR(34) &amp; ": " &amp; CHAR(34) &amp; E30 &amp; CHAR(34) &amp; CHAR(10)&amp; "      }" &amp; CHAR(10)&amp; "    }" &amp; CHAR(10)&amp; "  }" &amp; CHAR(10)&amp; "}")</f>
         <v/>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" s="34"/>
-    <row r="46" ht="36" customHeight="1" s="34">
-      <c r="A46" s="65" t="n"/>
-      <c r="B46" s="66" t="inlineStr">
+    <row r="46" ht="36" customHeight="1" s="34"/>
+    <row r="47">
+      <c r="A47" s="65" t="n"/>
+      <c r="B47" s="66" t="inlineStr">
         <is>
           <t>⚠  This file contains secrets. Your Secret Key grants full database access. Store this file securely and never share it.</t>
         </is>
       </c>
-      <c r="F46" s="65" t="n"/>
+      <c r="F47" s="65" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
Fix tracker row heights after provider fields
</commit_message>
<xml_diff>
--- a/docs/open-brain-credential-tracker.xlsx
+++ b/docs/open-brain-credential-tracker.xlsx
@@ -287,7 +287,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -486,6 +486,12 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1080,17 +1086,17 @@
       </c>
       <c r="E26" s="47" t="n"/>
     </row>
-    <row r="27" ht="31.5" customHeight="1" s="34"/>
-    <row r="28" ht="21.75" customHeight="1" s="34">
-      <c r="A28" s="57" t="n"/>
-      <c r="B28" s="58" t="inlineStr">
+    <row r="27" ht="7.5" customHeight="1" s="34"/>
+    <row r="28" ht="31.5" customHeight="1" s="34">
+      <c r="A28" s="48" t="n"/>
+      <c r="B28" s="49" t="inlineStr">
         <is>
           <t>STEP 5 — CREATE AN ACCESS KEY</t>
         </is>
       </c>
-      <c r="F28" s="57" t="n"/>
-    </row>
-    <row r="29" ht="30" customHeight="1" s="34">
+      <c r="F28" s="48" t="n"/>
+    </row>
+    <row r="29" ht="21.75" customHeight="1" s="34">
       <c r="B29" s="42" t="inlineStr">
         <is>
           <t>Step</t>
@@ -1112,7 +1118,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="7.5" customHeight="1" s="34">
+    <row r="30" ht="30" customHeight="1" s="34">
       <c r="B30" s="44" t="inlineStr">
         <is>
           <t>5</t>
@@ -1130,17 +1136,17 @@
       </c>
       <c r="E30" s="47" t="n"/>
     </row>
-    <row r="31" ht="31.5" customHeight="1" s="34"/>
-    <row r="32" ht="21.75" customHeight="1" s="34">
-      <c r="A32" s="59" t="n"/>
-      <c r="B32" s="60" t="inlineStr">
+    <row r="31" ht="7.5" customHeight="1" s="34"/>
+    <row r="32" ht="31.5" customHeight="1" s="34">
+      <c r="A32" s="48" t="n"/>
+      <c r="B32" s="49" t="inlineStr">
         <is>
           <t>STEP 6 — DEPLOY THE MCP SERVER</t>
         </is>
       </c>
-      <c r="F32" s="59" t="n"/>
-    </row>
-    <row r="33" ht="30" customHeight="1" s="34">
+      <c r="F32" s="48" t="n"/>
+    </row>
+    <row r="33" ht="21.75" customHeight="1" s="34">
       <c r="B33" s="42" t="inlineStr">
         <is>
           <t>Step</t>
@@ -1231,7 +1237,7 @@
           <t>6.7</t>
         </is>
       </c>
-      <c r="C37" s="53" t="inlineStr">
+      <c r="C37" s="61" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
@@ -1241,18 +1247,18 @@
           <t>MCP Server URL</t>
         </is>
       </c>
-      <c r="E37" s="54">
+      <c r="E37" s="62">
         <f>IF(E11="","← enter Project Ref in Step 1","https://"&amp;E11&amp;".supabase.co/functions/v1/open-brain-mcp")</f>
         <v/>
       </c>
     </row>
-    <row r="38" ht="7.5" customHeight="1" s="34">
+    <row r="38" ht="30" customHeight="1" s="34">
       <c r="B38" s="44" t="inlineStr">
         <is>
           <t>6.7</t>
         </is>
       </c>
-      <c r="C38" s="53" t="inlineStr">
+      <c r="C38" s="61" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
@@ -1262,22 +1268,22 @@
           <t>MCP Connection URL</t>
         </is>
       </c>
-      <c r="E38" s="54">
+      <c r="E38" s="62">
         <f>IF(OR(E11="",E30=""),"← enter Project Ref + Access Key","https://"&amp;E11&amp;".supabase.co/functions/v1/open-brain-mcp?key="&amp;E30)</f>
         <v/>
       </c>
     </row>
-    <row r="39" ht="31.5" customHeight="1" s="34"/>
-    <row r="40" ht="21.75" customHeight="1" s="34">
-      <c r="A40" s="63" t="n"/>
-      <c r="B40" s="64" t="inlineStr">
+    <row r="39" ht="7.5" customHeight="1" s="34"/>
+    <row r="40" ht="31.5" customHeight="1" s="34">
+      <c r="A40" s="48" t="n"/>
+      <c r="B40" s="49" t="inlineStr">
         <is>
           <t>STEP 7 — CONNECT TO YOUR AI</t>
         </is>
       </c>
-      <c r="F40" s="63" t="n"/>
-    </row>
-    <row r="41" ht="30" customHeight="1" s="34">
+      <c r="F40" s="48" t="n"/>
+    </row>
+    <row r="41" ht="21.75" customHeight="1" s="34">
       <c r="B41" s="42" t="inlineStr">
         <is>
           <t>Step</t>
@@ -1320,7 +1326,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="36" customHeight="1" s="34">
+    <row r="43" ht="30" customHeight="1" s="34">
       <c r="B43" s="44" t="inlineStr">
         <is>
           <t>7.2</t>
@@ -1341,7 +1347,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="219.75" customHeight="1" s="34">
+    <row r="44" ht="36" customHeight="1" s="34">
       <c r="B44" s="44" t="inlineStr">
         <is>
           <t>7.3</t>
@@ -1357,12 +1363,12 @@
           <t>Terminal: Claude Code CLI command</t>
         </is>
       </c>
-      <c r="E44" s="62">
+      <c r="E44" s="67">
         <f>IF(OR(E11="",E30=""),"← enter Project Ref + Access Key","claude mcp add --transport http open-brain https://"&amp;E11&amp;".supabase.co/functions/v1/open-brain-mcp --header "&amp;CHAR(34)&amp;"x-brain-key: "&amp;E30&amp;CHAR(34))</f>
         <v/>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" s="34">
+    <row r="45" ht="219.75" customHeight="1" s="34">
       <c r="B45" s="44" t="inlineStr">
         <is>
           <t>7.4</t>
@@ -1373,13 +1379,13 @@
           <t>COPY</t>
         </is>
       </c>
-      <c r="D45" s="46" t="inlineStr">
+      <c r="D45" s="68" t="inlineStr">
         <is>
           <t>JSON config for mcp-remote clients
 (Cursor, VS Code, Windsurf)</t>
         </is>
       </c>
-      <c r="E45" s="62">
+      <c r="E45" s="67">
         <f>IF(OR(E11="",E30=""),"← enter Project Ref + Access Key","{" &amp; CHAR(10)&amp; "  " &amp; CHAR(34) &amp; "mcpServers" &amp; CHAR(34) &amp; ": {" &amp; CHAR(10)&amp; "    " &amp; CHAR(34) &amp; "open-brain" &amp; CHAR(34) &amp; ": {" &amp; CHAR(10)&amp; "      " &amp; CHAR(34) &amp; "command" &amp; CHAR(34) &amp; ": " &amp; CHAR(34) &amp; "npx" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "      " &amp; CHAR(34) &amp; "args" &amp; CHAR(34) &amp; ": [" &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "mcp-remote" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "https://" &amp; E11 &amp; ".supabase.co/functions/v1/open-brain-mcp" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "--header" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "x-brain-key:${BRAIN_KEY}" &amp; CHAR(34) &amp; CHAR(10)&amp; "      ]," &amp; CHAR(10)&amp; "      " &amp; CHAR(34) &amp; "env" &amp; CHAR(34) &amp; ": {" &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "BRAIN_KEY" &amp; CHAR(34) &amp; ": " &amp; CHAR(34) &amp; E30 &amp; CHAR(34) &amp; CHAR(10)&amp; "      }" &amp; CHAR(10)&amp; "    }" &amp; CHAR(10)&amp; "  }" &amp; CHAR(10)&amp; "}")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Fix PR gate and tracker formatting
</commit_message>
<xml_diff>
--- a/docs/open-brain-credential-tracker.xlsx
+++ b/docs/open-brain-credential-tracker.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -136,8 +136,20 @@
       <color rgb="FFCC3333"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFCC3333"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -220,6 +232,31 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF0F0"/>
         <bgColor rgb="FFEEEEEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF43A047"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00897B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E88E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5C6BC0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF0F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -287,7 +324,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -451,22 +488,25 @@
     <xf numFmtId="0" fontId="14" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -475,23 +515,11 @@
     <xf numFmtId="0" fontId="15" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -985,7 +1013,7 @@
     <row r="20" ht="7.5" customHeight="1" s="34"/>
     <row r="21" ht="31.5" customHeight="1" s="34">
       <c r="A21" s="55" t="n"/>
-      <c r="B21" s="56" t="inlineStr">
+      <c r="B21" s="55" t="inlineStr">
         <is>
           <t>STEP 4 — GET AN AI API KEY</t>
         </is>
@@ -1015,22 +1043,22 @@
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" s="34">
-      <c r="B23" s="44" t="inlineStr">
+      <c r="B23" s="56" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C23" s="45" t="inlineStr">
+      <c r="C23" s="57" t="inlineStr">
         <is>
           <t>ENTER</t>
         </is>
       </c>
-      <c r="D23" s="46" t="inlineStr">
+      <c r="D23" s="58" t="inlineStr">
         <is>
           <t>AI Provider (OpenRouter or OpenAI)</t>
         </is>
       </c>
-      <c r="E23" s="47" t="n"/>
+      <c r="E23" s="59" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1" s="34">
       <c r="B24" s="44" t="inlineStr">
@@ -1086,15 +1114,15 @@
       </c>
       <c r="E26" s="47" t="n"/>
     </row>
-    <row r="27" ht="7.5" customHeight="1" s="34"/>
+    <row r="27" ht="8" customHeight="1" s="34"/>
     <row r="28" ht="31.5" customHeight="1" s="34">
-      <c r="A28" s="48" t="n"/>
-      <c r="B28" s="49" t="inlineStr">
+      <c r="A28" s="60" t="n"/>
+      <c r="B28" s="60" t="inlineStr">
         <is>
           <t>STEP 5 — CREATE AN ACCESS KEY</t>
         </is>
       </c>
-      <c r="F28" s="48" t="n"/>
+      <c r="F28" s="60" t="n"/>
     </row>
     <row r="29" ht="21.75" customHeight="1" s="34">
       <c r="B29" s="42" t="inlineStr">
@@ -1136,15 +1164,15 @@
       </c>
       <c r="E30" s="47" t="n"/>
     </row>
-    <row r="31" ht="7.5" customHeight="1" s="34"/>
+    <row r="31" ht="8" customHeight="1" s="34"/>
     <row r="32" ht="31.5" customHeight="1" s="34">
-      <c r="A32" s="48" t="n"/>
-      <c r="B32" s="49" t="inlineStr">
+      <c r="A32" s="61" t="n"/>
+      <c r="B32" s="61" t="inlineStr">
         <is>
           <t>STEP 6 — DEPLOY THE MCP SERVER</t>
         </is>
       </c>
-      <c r="F32" s="48" t="n"/>
+      <c r="F32" s="61" t="n"/>
     </row>
     <row r="33" ht="21.75" customHeight="1" s="34">
       <c r="B33" s="42" t="inlineStr">
@@ -1174,7 +1202,7 @@
           <t>6.4</t>
         </is>
       </c>
-      <c r="C34" s="61" t="inlineStr">
+      <c r="C34" s="62" t="inlineStr">
         <is>
           <t>COPY</t>
         </is>
@@ -1184,7 +1212,7 @@
           <t>Terminal: supabase link command</t>
         </is>
       </c>
-      <c r="E34" s="62">
+      <c r="E34" s="63">
         <f>IF(E11="","← enter Project Ref in Step 1","supabase link --project-ref "&amp;E11)</f>
         <v/>
       </c>
@@ -1195,7 +1223,7 @@
           <t>6.5</t>
         </is>
       </c>
-      <c r="C35" s="61" t="inlineStr">
+      <c r="C35" s="62" t="inlineStr">
         <is>
           <t>COPY</t>
         </is>
@@ -1205,7 +1233,7 @@
           <t>Terminal: set MCP Access Key secret</t>
         </is>
       </c>
-      <c r="E35" s="62">
+      <c r="E35" s="63">
         <f>IF(E30="","← enter Access Key in Step 5","supabase secrets set MCP_ACCESS_KEY="&amp;E30)</f>
         <v/>
       </c>
@@ -1216,7 +1244,7 @@
           <t>6.5</t>
         </is>
       </c>
-      <c r="C36" s="61" t="inlineStr">
+      <c r="C36" s="62" t="inlineStr">
         <is>
           <t>COPY</t>
         </is>
@@ -1226,7 +1254,7 @@
           <t>Terminal: set AI API Key secret</t>
         </is>
       </c>
-      <c r="E36" s="62">
+      <c r="E36" s="63">
         <f>IF(E26="","← enter AI API Key in Step 4",IF(E23="","← enter Provider in Step 4",IF(ISNUMBER(SEARCH("openai",LOWER(E23))),"supabase secrets set OPENAI_API_KEY="&amp;E26,"supabase secrets set OPENROUTER_API_KEY="&amp;E26)))</f>
         <v/>
       </c>
@@ -1237,7 +1265,7 @@
           <t>6.7</t>
         </is>
       </c>
-      <c r="C37" s="61" t="inlineStr">
+      <c r="C37" s="53" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
@@ -1247,7 +1275,7 @@
           <t>MCP Server URL</t>
         </is>
       </c>
-      <c r="E37" s="62">
+      <c r="E37" s="54">
         <f>IF(E11="","← enter Project Ref in Step 1","https://"&amp;E11&amp;".supabase.co/functions/v1/open-brain-mcp")</f>
         <v/>
       </c>
@@ -1258,7 +1286,7 @@
           <t>6.7</t>
         </is>
       </c>
-      <c r="C38" s="61" t="inlineStr">
+      <c r="C38" s="53" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
@@ -1268,20 +1296,20 @@
           <t>MCP Connection URL</t>
         </is>
       </c>
-      <c r="E38" s="62">
+      <c r="E38" s="54">
         <f>IF(OR(E11="",E30=""),"← enter Project Ref + Access Key","https://"&amp;E11&amp;".supabase.co/functions/v1/open-brain-mcp?key="&amp;E30)</f>
         <v/>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" s="34"/>
+    <row r="39" ht="8" customHeight="1" s="34"/>
     <row r="40" ht="31.5" customHeight="1" s="34">
-      <c r="A40" s="48" t="n"/>
-      <c r="B40" s="49" t="inlineStr">
+      <c r="A40" s="64" t="n"/>
+      <c r="B40" s="64" t="inlineStr">
         <is>
           <t>STEP 7 — CONNECT TO YOUR AI</t>
         </is>
       </c>
-      <c r="F40" s="48" t="n"/>
+      <c r="F40" s="64" t="n"/>
     </row>
     <row r="41" ht="21.75" customHeight="1" s="34">
       <c r="B41" s="42" t="inlineStr">
@@ -1311,7 +1339,7 @@
           <t>7.1</t>
         </is>
       </c>
-      <c r="C42" s="61" t="inlineStr">
+      <c r="C42" s="62" t="inlineStr">
         <is>
           <t>COPY</t>
         </is>
@@ -1321,7 +1349,7 @@
           <t>Claude Desktop → Connectors → Remote MCP server URL</t>
         </is>
       </c>
-      <c r="E42" s="62">
+      <c r="E42" s="63">
         <f>E38</f>
         <v/>
       </c>
@@ -1332,7 +1360,7 @@
           <t>7.2</t>
         </is>
       </c>
-      <c r="C43" s="61" t="inlineStr">
+      <c r="C43" s="62" t="inlineStr">
         <is>
           <t>COPY</t>
         </is>
@@ -1342,7 +1370,7 @@
           <t>ChatGPT → Apps &amp; Connectors → MCP endpoint URL</t>
         </is>
       </c>
-      <c r="E43" s="62">
+      <c r="E43" s="63">
         <f>E38</f>
         <v/>
       </c>
@@ -1353,7 +1381,7 @@
           <t>7.3</t>
         </is>
       </c>
-      <c r="C44" s="61" t="inlineStr">
+      <c r="C44" s="62" t="inlineStr">
         <is>
           <t>COPY</t>
         </is>
@@ -1363,7 +1391,7 @@
           <t>Terminal: Claude Code CLI command</t>
         </is>
       </c>
-      <c r="E44" s="67">
+      <c r="E44" s="63">
         <f>IF(OR(E11="",E30=""),"← enter Project Ref + Access Key","claude mcp add --transport http open-brain https://"&amp;E11&amp;".supabase.co/functions/v1/open-brain-mcp --header "&amp;CHAR(34)&amp;"x-brain-key: "&amp;E30&amp;CHAR(34))</f>
         <v/>
       </c>
@@ -1374,26 +1402,26 @@
           <t>7.4</t>
         </is>
       </c>
-      <c r="C45" s="61" t="inlineStr">
+      <c r="C45" s="62" t="inlineStr">
         <is>
           <t>COPY</t>
         </is>
       </c>
-      <c r="D45" s="68" t="inlineStr">
+      <c r="D45" s="46" t="inlineStr">
         <is>
           <t>JSON config for mcp-remote clients
 (Cursor, VS Code, Windsurf)</t>
         </is>
       </c>
-      <c r="E45" s="67">
+      <c r="E45" s="63">
         <f>IF(OR(E11="",E30=""),"← enter Project Ref + Access Key","{" &amp; CHAR(10)&amp; "  " &amp; CHAR(34) &amp; "mcpServers" &amp; CHAR(34) &amp; ": {" &amp; CHAR(10)&amp; "    " &amp; CHAR(34) &amp; "open-brain" &amp; CHAR(34) &amp; ": {" &amp; CHAR(10)&amp; "      " &amp; CHAR(34) &amp; "command" &amp; CHAR(34) &amp; ": " &amp; CHAR(34) &amp; "npx" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "      " &amp; CHAR(34) &amp; "args" &amp; CHAR(34) &amp; ": [" &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "mcp-remote" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "https://" &amp; E11 &amp; ".supabase.co/functions/v1/open-brain-mcp" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "--header" &amp; CHAR(34) &amp; "," &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "x-brain-key:${BRAIN_KEY}" &amp; CHAR(34) &amp; CHAR(10)&amp; "      ]," &amp; CHAR(10)&amp; "      " &amp; CHAR(34) &amp; "env" &amp; CHAR(34) &amp; ": {" &amp; CHAR(10)&amp; "        " &amp; CHAR(34) &amp; "BRAIN_KEY" &amp; CHAR(34) &amp; ": " &amp; CHAR(34) &amp; E30 &amp; CHAR(34) &amp; CHAR(10)&amp; "      }" &amp; CHAR(10)&amp; "    }" &amp; CHAR(10)&amp; "  }" &amp; CHAR(10)&amp; "}")</f>
         <v/>
       </c>
     </row>
-    <row r="46" ht="36" customHeight="1" s="34"/>
-    <row r="47">
+    <row r="46" ht="8" customHeight="1" s="34"/>
+    <row r="47" ht="36" customHeight="1" s="34">
       <c r="A47" s="65" t="n"/>
-      <c r="B47" s="66" t="inlineStr">
+      <c r="B47" s="65" t="inlineStr">
         <is>
           <t>⚠  This file contains secrets. Your Secret Key grants full database access. Store this file securely and never share it.</t>
         </is>
@@ -1402,18 +1430,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B40:E40"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B13:E13"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B39:E39"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="B28:E28"/>
     <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B32:E32"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>